<commit_message>
Documentation update (chapters 5.3 and 5.5).
git-svn-id: https://scm.projects.hlrs.de/authscm/sleyh/svn/ms2@456 a2be33b2-7eaf-4dce-bf61-b02fde6c56c2
</commit_message>
<xml_diff>
--- a/documentation/Inhalt manual.xlsx
+++ b/documentation/Inhalt manual.xlsx
@@ -9,12 +9,12 @@
   <sheets>
     <sheet name="Outline" sheetId="3" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="145621"/>
+  <calcPr calcId="144525"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="98">
   <si>
     <t>1. Getting Started</t>
   </si>
@@ -106,12 +106,6 @@
     <t>Sammeln</t>
   </si>
   <si>
-    <t>(Gabor)?</t>
-  </si>
-  <si>
-    <t>(Gabor) ?</t>
-  </si>
-  <si>
     <t>hlrs</t>
   </si>
   <si>
@@ -175,9 +169,6 @@
     <t>5.3 Monte Carlo</t>
   </si>
   <si>
-    <t>5.3.1 Moves</t>
-  </si>
-  <si>
     <t>5.3.2 Resize</t>
   </si>
   <si>
@@ -311,6 +302,12 @@
   </si>
   <si>
     <t>Stand</t>
+  </si>
+  <si>
+    <t>Gabor</t>
+  </si>
+  <si>
+    <t>5.3.1 Translation and rotation</t>
   </si>
 </sst>
 </file>
@@ -423,9 +420,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -458,22 +452,25 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -786,60 +783,60 @@
     <col min="2" max="2" width="9.140625" style="3"/>
     <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.5703125" customWidth="1"/>
-    <col min="6" max="6" width="15.5703125" style="26" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.5703125" style="24" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:9" s="20" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A2" s="21"/>
-      <c r="B2" s="21"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="23" t="s">
-        <v>97</v>
-      </c>
-      <c r="G2" s="22" t="s">
-        <v>98</v>
-      </c>
-      <c r="H2" s="22"/>
-      <c r="I2" s="22"/>
+    <row r="2" spans="1:9" s="19" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A2" s="20"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="22" t="s">
+        <v>94</v>
+      </c>
+      <c r="G2" s="21" t="s">
+        <v>95</v>
+      </c>
+      <c r="H2" s="21"/>
+      <c r="I2" s="21"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="F3" s="24" t="s">
+        <v>43</v>
+      </c>
+      <c r="F3" s="27" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="F4" s="24"/>
+        <v>44</v>
+      </c>
+      <c r="F4" s="27"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="F5" s="24"/>
+        <v>45</v>
+      </c>
+      <c r="F5" s="27"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="F6" s="25"/>
+      <c r="F6" s="23"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="F7" s="25" t="s">
+      <c r="F7" s="23" t="s">
         <v>20</v>
       </c>
     </row>
@@ -847,15 +844,15 @@
       <c r="B8" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F8" s="24" t="s">
-        <v>32</v>
+      <c r="F8" s="27" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F9" s="24"/>
+      <c r="F9" s="27"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
@@ -866,7 +863,7 @@
       <c r="B11" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F11" s="24" t="s">
+      <c r="F11" s="27" t="s">
         <v>20</v>
       </c>
     </row>
@@ -874,43 +871,43 @@
       <c r="B12" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F12" s="24"/>
+      <c r="F12" s="27"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B13" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F13" s="24"/>
+      <c r="F13" s="27"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B14" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F14" s="24"/>
+      <c r="F14" s="27"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B15" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F15" s="24"/>
+      <c r="F15" s="27"/>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B16" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F16" s="24"/>
+      <c r="F16" s="27"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B17" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F17" s="24"/>
+      <c r="F17" s="27"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F18" s="24" t="s">
+      <c r="F18" s="27" t="s">
         <v>21</v>
       </c>
     </row>
@@ -918,19 +915,19 @@
       <c r="B19" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F19" s="24"/>
+      <c r="F19" s="27"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B20" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F20" s="24"/>
+      <c r="F20" s="27"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B21" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F21" s="24"/>
+      <c r="F21" s="27"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
@@ -940,119 +937,119 @@
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
       <c r="B23" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="F23" s="26" t="s">
+        <v>46</v>
+      </c>
+      <c r="F23" s="24" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B24" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="F24" s="24" t="s">
+        <v>47</v>
+      </c>
+      <c r="F24" s="27" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C25" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="F25" s="24"/>
+        <v>48</v>
+      </c>
+      <c r="F25" s="27"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C26" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="F26" s="24"/>
+        <v>49</v>
+      </c>
+      <c r="F26" s="27"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B27" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="F27" s="24" t="s">
-        <v>30</v>
+        <v>50</v>
+      </c>
+      <c r="F27" s="27" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C28" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="F28" s="24"/>
+        <v>97</v>
+      </c>
+      <c r="F28" s="27"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C29" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F29" s="24"/>
+        <v>51</v>
+      </c>
+      <c r="F29" s="27"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B30" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="F30" s="26" t="s">
+        <v>52</v>
+      </c>
+      <c r="F30" s="24" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B31" s="2" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C32" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="F32" s="27" t="s">
+        <v>54</v>
+      </c>
+      <c r="F32" s="30" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C33" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="F33" s="27"/>
+        <v>55</v>
+      </c>
+      <c r="F33" s="30"/>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C34" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="F34" s="27"/>
+        <v>56</v>
+      </c>
+      <c r="F34" s="30"/>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C35" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="F35" s="27"/>
+        <v>57</v>
+      </c>
+      <c r="F35" s="30"/>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C36" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="F36" s="27"/>
+        <v>58</v>
+      </c>
+      <c r="F36" s="30"/>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B37" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C38" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="F38" s="26" t="s">
+        <v>60</v>
+      </c>
+      <c r="F38" s="24" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A39" s="13"/>
-      <c r="B39" s="13"/>
-      <c r="C39" s="14" t="s">
-        <v>64</v>
+      <c r="A39" s="12"/>
+      <c r="B39" s="12"/>
+      <c r="C39" s="13" t="s">
+        <v>61</v>
       </c>
       <c r="D39" s="4"/>
       <c r="E39" s="4"/>
-      <c r="F39" s="28" t="s">
+      <c r="F39" s="25" t="s">
         <v>27</v>
       </c>
       <c r="G39" s="4"/>
@@ -1062,14 +1059,14 @@
       <c r="K39" s="4"/>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A40" s="13"/>
-      <c r="B40" s="13"/>
-      <c r="C40" s="14" t="s">
-        <v>65</v>
+      <c r="A40" s="12"/>
+      <c r="B40" s="12"/>
+      <c r="C40" s="13" t="s">
+        <v>62</v>
       </c>
       <c r="D40" s="4"/>
       <c r="E40" s="4"/>
-      <c r="F40" s="28" t="s">
+      <c r="F40" s="25" t="s">
         <v>22</v>
       </c>
       <c r="G40" s="4"/>
@@ -1079,14 +1076,14 @@
       <c r="K40" s="4"/>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A41" s="13"/>
-      <c r="B41" s="13"/>
-      <c r="C41" s="14" t="s">
-        <v>66</v>
+      <c r="A41" s="12"/>
+      <c r="B41" s="12"/>
+      <c r="C41" s="13" t="s">
+        <v>63</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4"/>
-      <c r="F41" s="28" t="s">
+      <c r="F41" s="25" t="s">
         <v>20</v>
       </c>
       <c r="G41" s="4"/>
@@ -1096,14 +1093,14 @@
       <c r="K41" s="4"/>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A42" s="13"/>
-      <c r="B42" s="14" t="s">
-        <v>67</v>
+      <c r="A42" s="12"/>
+      <c r="B42" s="13" t="s">
+        <v>64</v>
       </c>
       <c r="C42" s="4"/>
       <c r="D42" s="4"/>
       <c r="E42" s="4"/>
-      <c r="F42" s="29" t="s">
+      <c r="F42" s="28" t="s">
         <v>21</v>
       </c>
       <c r="G42" s="4"/>
@@ -1113,14 +1110,14 @@
       <c r="K42" s="4"/>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A43" s="13"/>
-      <c r="B43" s="13"/>
-      <c r="C43" s="14" t="s">
-        <v>68</v>
+      <c r="A43" s="12"/>
+      <c r="B43" s="12"/>
+      <c r="C43" s="13" t="s">
+        <v>65</v>
       </c>
       <c r="D43" s="4"/>
       <c r="E43" s="4"/>
-      <c r="F43" s="29"/>
+      <c r="F43" s="28"/>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
       <c r="I43" s="4"/>
@@ -1128,14 +1125,14 @@
       <c r="K43" s="4"/>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A44" s="13"/>
-      <c r="B44" s="13"/>
-      <c r="C44" s="14" t="s">
-        <v>69</v>
+      <c r="A44" s="12"/>
+      <c r="B44" s="12"/>
+      <c r="C44" s="13" t="s">
+        <v>66</v>
       </c>
       <c r="D44" s="4"/>
       <c r="E44" s="4"/>
-      <c r="F44" s="29"/>
+      <c r="F44" s="28"/>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
       <c r="I44" s="4"/>
@@ -1143,14 +1140,14 @@
       <c r="K44" s="4"/>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A45" s="13"/>
-      <c r="B45" s="14" t="s">
-        <v>73</v>
+      <c r="A45" s="12"/>
+      <c r="B45" s="13" t="s">
+        <v>70</v>
       </c>
       <c r="C45" s="4"/>
       <c r="D45" s="4"/>
       <c r="E45" s="4"/>
-      <c r="F45" s="28"/>
+      <c r="F45" s="25"/>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
       <c r="I45" s="4"/>
@@ -1158,14 +1155,14 @@
       <c r="K45" s="4"/>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A46" s="13"/>
-      <c r="B46" s="13"/>
-      <c r="C46" s="14" t="s">
-        <v>72</v>
+      <c r="A46" s="12"/>
+      <c r="B46" s="12"/>
+      <c r="C46" s="13" t="s">
+        <v>69</v>
       </c>
       <c r="D46" s="4"/>
       <c r="E46" s="4"/>
-      <c r="F46" s="28" t="s">
+      <c r="F46" s="25" t="s">
         <v>22</v>
       </c>
       <c r="G46" s="4"/>
@@ -1175,15 +1172,15 @@
       <c r="K46" s="4"/>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A47" s="13"/>
-      <c r="B47" s="13"/>
-      <c r="C47" s="14" t="s">
-        <v>71</v>
+      <c r="A47" s="12"/>
+      <c r="B47" s="12"/>
+      <c r="C47" s="13" t="s">
+        <v>68</v>
       </c>
       <c r="D47" s="4"/>
       <c r="E47" s="4"/>
-      <c r="F47" s="28" t="s">
-        <v>31</v>
+      <c r="F47" s="25" t="s">
+        <v>96</v>
       </c>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -1192,15 +1189,15 @@
       <c r="K47" s="4"/>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A48" s="13"/>
-      <c r="B48" s="13"/>
-      <c r="C48" s="14" t="s">
-        <v>70</v>
+      <c r="A48" s="12"/>
+      <c r="B48" s="12"/>
+      <c r="C48" s="13" t="s">
+        <v>67</v>
       </c>
       <c r="D48" s="4"/>
       <c r="E48" s="4"/>
-      <c r="F48" s="28" t="s">
-        <v>31</v>
+      <c r="F48" s="25" t="s">
+        <v>96</v>
       </c>
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
@@ -1209,14 +1206,14 @@
       <c r="K48" s="4"/>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A49" s="13"/>
-      <c r="B49" s="13"/>
-      <c r="C49" s="14" t="s">
-        <v>74</v>
+      <c r="A49" s="12"/>
+      <c r="B49" s="12"/>
+      <c r="C49" s="13" t="s">
+        <v>71</v>
       </c>
       <c r="D49" s="4"/>
       <c r="E49" s="4"/>
-      <c r="F49" s="28" t="s">
+      <c r="F49" s="25" t="s">
         <v>24</v>
       </c>
       <c r="G49" s="4"/>
@@ -1226,15 +1223,15 @@
       <c r="K49" s="4"/>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A50" s="13"/>
-      <c r="B50" s="13"/>
-      <c r="C50" s="14" t="s">
-        <v>75</v>
+      <c r="A50" s="12"/>
+      <c r="B50" s="12"/>
+      <c r="C50" s="13" t="s">
+        <v>72</v>
       </c>
       <c r="D50" s="4"/>
       <c r="E50" s="4"/>
-      <c r="F50" s="28" t="s">
-        <v>94</v>
+      <c r="F50" s="25" t="s">
+        <v>91</v>
       </c>
       <c r="G50" s="4"/>
       <c r="H50" s="4"/>
@@ -1243,14 +1240,14 @@
       <c r="K50" s="4"/>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A51" s="13"/>
-      <c r="B51" s="13"/>
-      <c r="C51" s="15" t="s">
-        <v>76</v>
+      <c r="A51" s="12"/>
+      <c r="B51" s="12"/>
+      <c r="C51" s="14" t="s">
+        <v>73</v>
       </c>
       <c r="D51" s="4"/>
       <c r="E51" s="4"/>
-      <c r="F51" s="28"/>
+      <c r="F51" s="25"/>
       <c r="G51" s="4"/>
       <c r="H51" s="4"/>
       <c r="I51" s="4"/>
@@ -1258,14 +1255,14 @@
       <c r="K51" s="4"/>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A52" s="13"/>
-      <c r="B52" s="13"/>
-      <c r="C52" s="14" t="s">
-        <v>77</v>
+      <c r="A52" s="12"/>
+      <c r="B52" s="12"/>
+      <c r="C52" s="13" t="s">
+        <v>74</v>
       </c>
       <c r="D52" s="4"/>
       <c r="E52" s="4"/>
-      <c r="F52" s="28"/>
+      <c r="F52" s="25"/>
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
       <c r="I52" s="4"/>
@@ -1273,14 +1270,14 @@
       <c r="K52" s="4"/>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A53" s="13"/>
-      <c r="B53" s="14" t="s">
-        <v>78</v>
+      <c r="A53" s="12"/>
+      <c r="B53" s="13" t="s">
+        <v>75</v>
       </c>
       <c r="C53" s="4"/>
       <c r="D53" s="4"/>
       <c r="E53" s="4"/>
-      <c r="F53" s="28" t="s">
+      <c r="F53" s="25" t="s">
         <v>21</v>
       </c>
       <c r="G53" s="4"/>
@@ -1290,14 +1287,14 @@
       <c r="K53" s="4"/>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A54" s="13"/>
-      <c r="B54" s="14" t="s">
-        <v>95</v>
+      <c r="A54" s="12"/>
+      <c r="B54" s="13" t="s">
+        <v>92</v>
       </c>
       <c r="C54" s="4"/>
       <c r="D54" s="4"/>
       <c r="E54" s="4"/>
-      <c r="F54" s="28"/>
+      <c r="F54" s="25"/>
       <c r="G54" s="4"/>
       <c r="H54" s="4"/>
       <c r="I54" s="4"/>
@@ -1305,14 +1302,14 @@
       <c r="K54" s="4"/>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A55" s="13"/>
-      <c r="B55" s="13"/>
-      <c r="C55" s="14" t="s">
-        <v>79</v>
+      <c r="A55" s="12"/>
+      <c r="B55" s="12"/>
+      <c r="C55" s="13" t="s">
+        <v>76</v>
       </c>
       <c r="D55" s="4"/>
       <c r="E55" s="4"/>
-      <c r="F55" s="28" t="s">
+      <c r="F55" s="25" t="s">
         <v>28</v>
       </c>
       <c r="G55" s="4"/>
@@ -1322,15 +1319,15 @@
       <c r="K55" s="4"/>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A56" s="13"/>
-      <c r="B56" s="13"/>
-      <c r="C56" s="14" t="s">
-        <v>80</v>
+      <c r="A56" s="12"/>
+      <c r="B56" s="12"/>
+      <c r="C56" s="13" t="s">
+        <v>77</v>
       </c>
       <c r="D56" s="4"/>
       <c r="E56" s="4"/>
-      <c r="F56" s="28" t="s">
-        <v>93</v>
+      <c r="F56" s="25" t="s">
+        <v>90</v>
       </c>
       <c r="G56" s="4"/>
       <c r="H56" s="4"/>
@@ -1339,18 +1336,18 @@
       <c r="K56" s="4"/>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A57" s="13"/>
-      <c r="B57" s="13"/>
-      <c r="C57" s="16" t="s">
+      <c r="A57" s="12"/>
+      <c r="B57" s="12"/>
+      <c r="C57" s="15" t="s">
         <v>18</v>
       </c>
       <c r="D57" s="4"/>
       <c r="E57" s="4"/>
-      <c r="F57" s="28" t="s">
+      <c r="F57" s="25" t="s">
         <v>20</v>
       </c>
       <c r="G57" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="H57" s="4"/>
       <c r="I57" s="4"/>
@@ -1358,15 +1355,15 @@
       <c r="K57" s="4"/>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A58" s="13"/>
-      <c r="B58" s="13"/>
-      <c r="C58" s="14" t="s">
-        <v>81</v>
+      <c r="A58" s="12"/>
+      <c r="B58" s="12"/>
+      <c r="C58" s="13" t="s">
+        <v>78</v>
       </c>
       <c r="D58" s="4"/>
       <c r="E58" s="4"/>
-      <c r="F58" s="28" t="s">
-        <v>33</v>
+      <c r="F58" s="25" t="s">
+        <v>31</v>
       </c>
       <c r="G58" s="4"/>
       <c r="H58" s="4"/>
@@ -1375,15 +1372,15 @@
       <c r="K58" s="4"/>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A59" s="13"/>
-      <c r="B59" s="13"/>
-      <c r="C59" s="17" t="s">
-        <v>82</v>
+      <c r="A59" s="12"/>
+      <c r="B59" s="12"/>
+      <c r="C59" s="16" t="s">
+        <v>79</v>
       </c>
       <c r="D59" s="4"/>
       <c r="E59" s="4"/>
-      <c r="F59" s="28" t="s">
-        <v>33</v>
+      <c r="F59" s="25" t="s">
+        <v>31</v>
       </c>
       <c r="G59" s="4"/>
       <c r="H59" s="4"/>
@@ -1392,17 +1389,17 @@
       <c r="K59" s="4"/>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A60" s="18" t="s">
-        <v>36</v>
-      </c>
-      <c r="B60" s="13" t="s">
-        <v>37</v>
+      <c r="A60" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="B60" s="12" t="s">
+        <v>35</v>
       </c>
       <c r="C60" s="4"/>
-      <c r="D60" s="19"/>
+      <c r="D60" s="18"/>
       <c r="E60" s="4"/>
-      <c r="F60" s="28" t="s">
-        <v>44</v>
+      <c r="F60" s="25" t="s">
+        <v>42</v>
       </c>
       <c r="G60" s="4"/>
       <c r="H60" s="4"/>
@@ -1412,150 +1409,150 @@
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D61" s="5"/>
-      <c r="F61" s="25"/>
+      <c r="F61" s="23"/>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" s="7" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B62" s="8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C62" s="9"/>
       <c r="D62" s="10"/>
-      <c r="E62" s="11" t="s">
+      <c r="E62" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="F62" s="30"/>
+      <c r="F62" s="26"/>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" s="7"/>
       <c r="B63" s="8" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C63" s="9"/>
       <c r="D63" s="10"/>
-      <c r="E63" s="11"/>
-      <c r="F63" s="30"/>
+      <c r="E63" s="29"/>
+      <c r="F63" s="26"/>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" s="7"/>
       <c r="B64" s="8" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C64" s="9"/>
       <c r="D64" s="10"/>
-      <c r="E64" s="11"/>
-      <c r="F64" s="30"/>
+      <c r="E64" s="29"/>
+      <c r="F64" s="26"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="7"/>
       <c r="B65" s="8" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C65" s="9"/>
       <c r="D65" s="10"/>
-      <c r="E65" s="11"/>
-      <c r="F65" s="30"/>
+      <c r="E65" s="29"/>
+      <c r="F65" s="26"/>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="7"/>
       <c r="B66" s="8" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C66" s="9"/>
       <c r="D66" s="10"/>
-      <c r="E66" s="11"/>
-      <c r="F66" s="30" t="s">
-        <v>42</v>
+      <c r="E66" s="29"/>
+      <c r="F66" s="26" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="7" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B67" s="8"/>
       <c r="C67" s="9"/>
       <c r="D67" s="10"/>
-      <c r="E67" s="11"/>
-      <c r="F67" s="30"/>
+      <c r="E67" s="29"/>
+      <c r="F67" s="26"/>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="8"/>
-      <c r="B68" s="12" t="s">
-        <v>86</v>
+      <c r="B68" s="11" t="s">
+        <v>83</v>
       </c>
       <c r="C68" s="9"/>
       <c r="D68" s="10"/>
-      <c r="E68" s="11"/>
+      <c r="E68" s="29"/>
       <c r="F68" s="31" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="8"/>
-      <c r="B69" s="12" t="s">
-        <v>87</v>
+      <c r="B69" s="11" t="s">
+        <v>84</v>
       </c>
       <c r="C69" s="9"/>
       <c r="D69" s="10"/>
-      <c r="E69" s="11"/>
+      <c r="E69" s="29"/>
       <c r="F69" s="31"/>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="8"/>
-      <c r="B70" s="12" t="s">
-        <v>88</v>
+      <c r="B70" s="11" t="s">
+        <v>85</v>
       </c>
       <c r="C70" s="9"/>
       <c r="D70" s="10"/>
-      <c r="E70" s="11"/>
+      <c r="E70" s="29"/>
       <c r="F70" s="31"/>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="8"/>
-      <c r="B71" s="12" t="s">
-        <v>89</v>
+      <c r="B71" s="11" t="s">
+        <v>86</v>
       </c>
       <c r="C71" s="9"/>
       <c r="D71" s="10"/>
-      <c r="E71" s="11"/>
+      <c r="E71" s="29"/>
       <c r="F71" s="31"/>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="8"/>
-      <c r="B72" s="12" t="s">
-        <v>90</v>
+      <c r="B72" s="11" t="s">
+        <v>87</v>
       </c>
       <c r="C72" s="9"/>
       <c r="D72" s="10"/>
-      <c r="E72" s="11"/>
+      <c r="E72" s="29"/>
       <c r="F72" s="31"/>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="7" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B73" s="8"/>
       <c r="C73" s="9"/>
       <c r="D73" s="10"/>
-      <c r="E73" s="11"/>
-      <c r="F73" s="30" t="s">
-        <v>96</v>
+      <c r="E73" s="29"/>
+      <c r="F73" s="26" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" s="7" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B74" s="8"/>
       <c r="C74" s="9"/>
       <c r="D74" s="10"/>
-      <c r="E74" s="11"/>
-      <c r="F74" s="30" t="s">
+      <c r="E74" s="29"/>
+      <c r="F74" s="26" t="s">
         <v>26</v>
       </c>
     </row>
@@ -1566,20 +1563,20 @@
       <c r="B75" s="8"/>
       <c r="C75" s="9"/>
       <c r="D75" s="10"/>
-      <c r="E75" s="11"/>
-      <c r="F75" s="30" t="s">
+      <c r="E75" s="29"/>
+      <c r="F75" s="26" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" s="7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B76" s="8"/>
       <c r="C76" s="9"/>
       <c r="D76" s="10"/>
-      <c r="E76" s="11"/>
-      <c r="F76" s="30" t="s">
+      <c r="E76" s="29"/>
+      <c r="F76" s="26" t="s">
         <v>20</v>
       </c>
     </row>

</xml_diff>